<commit_message>
Stage 8 fixes: A-017
</commit_message>
<xml_diff>
--- a/output/archive/VellacombeData/Clients/EB05/VD-22-076/Delivery/LotB/EB05_resupply_24Oct22_v3_FINAL_final.xlsx
+++ b/output/archive/VellacombeData/Clients/EB05/VD-22-076/Delivery/LotB/EB05_resupply_24Oct22_v3_FINAL_final.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -442,121 +442,110 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Vellacombe Discovery Ltd, a Tarnovell company</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
           <t>VD-22-076 Elvarmere chiral intermediate resupply, campaign B</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>VD-22-076</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>LIMS</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>VA20220698</t>
+          <t>VD-22-076</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Client</t>
+          <t>LIMS</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Elvarmere Biosciences AB</t>
+          <t>VA20220698</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>Client</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>GBP 50,300</t>
+          <t>Elvarmere Biosciences AB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GBP 50,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Turnaround (days)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B7" s="3" t="n">
         <v>98</v>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Outcome</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Resupply met the enantiomeric-purity specification agreed at quote. Elvarmere's downstream synthesis restarted on release.</t>
-        </is>
-      </c>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Resupply met the enantiomeric-purity specification agreed at quote. Elvarmere's downstream synthesis restarted on release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Lot status</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Released. Measurements and isolated mass are on the Lot sheet; the release sign-off is on the Release sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Compiled by</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Clara Fenwick</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>24/10/2022</t>
-        </is>
-      </c>
-    </row>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Released. Numerical enantiomeric-purity measurements and isolated mass remain in the retained analytical run sheets and balance records under VA20220698; the Lot sheet links both sources to the same delivery lot. Release sign-off is on the Release sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Approved by</t>
+          <t>Compiled by</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Dr R. Calderwood</t>
+          <t>Clara Fenwick</t>
         </is>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -566,9 +555,28 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Approved by</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Dr R. Calderwood</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>24/10/2022</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -581,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -600,30 +608,30 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Enantiomeric purity by chiral HPLC on the method in the study plan. Isolated mass from the balance record, in g for the bulk lot.</t>
+          <t>Numerical chiral HPLC measurements and isolated mass remain in retained analytical and balance records under VA20220698. This workbook records the qualitative release outcome and source linkage, not transcribed measurements.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Measurement</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Delivery-lot item</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Analytical record reference</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Balance record reference</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Release outcome / note</t>
         </is>
       </c>
     </row>
@@ -635,17 +643,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chiral HPLC, enantiomeric purity</t>
+          <t>VA20220698: starting-material chiral HPLC run sheet</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Recorded on the run sheet</t>
+          <t>See campaign balance records</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Matches the lot sent for the resupply.</t>
+          <t>Starting-material identity linked to campaign B</t>
         </is>
       </c>
     </row>
@@ -657,74 +665,52 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Chiral HPLC, enantiomeric purity</t>
+          <t>VA20220698: intermediate chiral HPLC run sheet</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Recorded on the run sheet</t>
+          <t>See crystallisation balance record</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Second crystallisation was needed to reach the specification.</t>
+          <t>Second crystallisation required for specification</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bulk lot, final</t>
+          <t>Campaign B final delivery lot</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Chiral HPLC, enantiomeric purity</t>
+          <t>VA20220698: final-lot chiral HPLC run sheet</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Recorded on the run sheet</t>
+          <t>VA20220698: same final-lot isolated-mass balance record (g)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Within the agreed specification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Bulk lot, final</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Isolated mass</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Recorded on the balance record</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Handwritten mass transcribed here in g; checked by CF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+          <t>Met agreed enantiomeric-purity specification; approved for delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>The downstream synthesis at Elvarmere needs the isolated mass and the chiral result together. Keep both on the same line.</t>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Final delivery-lot chiral purity and isolated mass share the row above. Numerical values are retained only in linked source records.</t>
         </is>
       </c>
     </row>

</xml_diff>